<commit_message>
Add citation and contact sections, update to cleaned workbook
Adds a "Citing this work" section (APA + BibTeX) and a "Contact &
collaboration" section with LinkedIn/affiliation, matching the
byline pattern of the reference site. Replaces the assessment
workbook with the cleaned version (sample answers removed).
</commit_message>
<xml_diff>
--- a/assets/DSAF-Operational-Reversibility-v1.1.xlsx
+++ b/assets/DSAF-Operational-Reversibility-v1.1.xlsx
@@ -3,9 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB0CE150-5B3A-2C47-94BC-8BF92EC141FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zaynabmusawi/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14817A05-6939-B14F-AD33-6C0EC828F319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -67,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="466">
   <si>
     <t>Level</t>
   </si>
@@ -1672,9 +1677,6 @@
   <si>
     <t>→ Exit plan document (draft or otherwise); note: outdated or unapproved plans confirm M2.
 → Contract text showing absence of exit rights or presence of prohibitive exit fees.</t>
-  </si>
-  <si>
-    <t>✓</t>
   </si>
 </sst>
 </file>
@@ -2532,40 +2534,40 @@
     <xf numFmtId="0" fontId="0" fillId="27" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="45" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2578,17 +2580,56 @@
     <xf numFmtId="0" fontId="42" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="13" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2620,91 +2661,52 @@
     <xf numFmtId="0" fontId="28" fillId="14" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="15" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="16" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="21" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3097,36 +3099,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="70" t="s">
         <v>463</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="71" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
     </row>
     <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="72" t="s">
         <v>341</v>
       </c>
-      <c r="B4" s="63"/>
+      <c r="B4" s="72"/>
     </row>
     <row r="5" spans="1:3" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="68" t="s">
         <v>241</v>
       </c>
-      <c r="B5" s="67"/>
+      <c r="B5" s="69"/>
     </row>
     <row r="6" spans="1:3" ht="87" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="65" t="s">
+      <c r="A6" s="68" t="s">
         <v>323</v>
       </c>
-      <c r="B6" s="67"/>
+      <c r="B6" s="69"/>
     </row>
     <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="46" t="s">
@@ -3145,119 +3147,119 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="63" t="s">
+      <c r="A11" s="72" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="64"/>
+      <c r="B11" s="73"/>
     </row>
     <row r="12" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="65" t="s">
+      <c r="A12" s="68" t="s">
         <v>242</v>
       </c>
-      <c r="B12" s="66"/>
+      <c r="B12" s="74"/>
     </row>
     <row r="13" spans="1:3" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="65" t="s">
+      <c r="A13" s="68" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="67"/>
+      <c r="B13" s="69"/>
     </row>
     <row r="14" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="B14" s="67"/>
+      <c r="B14" s="69"/>
     </row>
     <row r="15" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="65" t="s">
+      <c r="A15" s="68" t="s">
         <v>431</v>
       </c>
-      <c r="B15" s="67"/>
+      <c r="B15" s="69"/>
     </row>
     <row r="17" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="72" t="s">
+      <c r="A17" s="65" t="s">
         <v>306</v>
       </c>
-      <c r="B17" s="72"/>
-      <c r="C17" s="72"/>
+      <c r="B17" s="65"/>
+      <c r="C17" s="65"/>
     </row>
     <row r="18" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="50" t="s">
         <v>308</v>
       </c>
-      <c r="B18" s="73" t="s">
+      <c r="B18" s="66" t="s">
         <v>315</v>
       </c>
-      <c r="C18" s="73"/>
+      <c r="C18" s="66"/>
     </row>
     <row r="19" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="50" t="s">
         <v>309</v>
       </c>
-      <c r="B19" s="73" t="s">
+      <c r="B19" s="66" t="s">
         <v>316</v>
       </c>
-      <c r="C19" s="73"/>
+      <c r="C19" s="66"/>
     </row>
     <row r="20" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="50" t="s">
         <v>310</v>
       </c>
-      <c r="B20" s="73" t="s">
+      <c r="B20" s="66" t="s">
         <v>321</v>
       </c>
-      <c r="C20" s="73"/>
+      <c r="C20" s="66"/>
     </row>
     <row r="21" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="50" t="s">
         <v>311</v>
       </c>
-      <c r="B21" s="73" t="s">
+      <c r="B21" s="66" t="s">
         <v>317</v>
       </c>
-      <c r="C21" s="73"/>
+      <c r="C21" s="66"/>
     </row>
     <row r="22" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="50" t="s">
         <v>312</v>
       </c>
-      <c r="B22" s="73" t="s">
+      <c r="B22" s="66" t="s">
         <v>318</v>
       </c>
-      <c r="C22" s="73"/>
+      <c r="C22" s="66"/>
     </row>
     <row r="23" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="50" t="s">
         <v>313</v>
       </c>
-      <c r="B23" s="73" t="s">
+      <c r="B23" s="66" t="s">
         <v>319</v>
       </c>
-      <c r="C23" s="73"/>
+      <c r="C23" s="66"/>
     </row>
     <row r="24" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="50" t="s">
         <v>314</v>
       </c>
-      <c r="B24" s="73" t="s">
+      <c r="B24" s="66" t="s">
         <v>320</v>
       </c>
-      <c r="C24" s="73"/>
+      <c r="C24" s="66"/>
     </row>
     <row r="25" spans="1:3" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="74" t="s">
+      <c r="A25" s="67" t="s">
         <v>307</v>
       </c>
-      <c r="B25" s="74"/>
-      <c r="C25" s="74"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
     </row>
     <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="70" t="s">
+      <c r="A27" s="63" t="s">
         <v>322</v>
       </c>
-      <c r="B27" s="71"/>
-      <c r="C27" s="71"/>
+      <c r="B27" s="64"/>
+      <c r="C27" s="64"/>
     </row>
     <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -3327,11 +3329,11 @@
     </row>
     <row r="34" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="71" t="s">
+      <c r="A35" s="64" t="s">
         <v>238</v>
       </c>
-      <c r="B35" s="71"/>
-      <c r="C35" s="71"/>
+      <c r="B35" s="64"/>
+      <c r="C35" s="64"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -3390,6 +3392,16 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A17:C17"/>
@@ -3401,16 +3413,6 @@
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3962,12 +3964,34 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A46:B46"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A56:B56"/>
@@ -3984,34 +4008,12 @@
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A52:B52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="94" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -4035,71 +4037,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="98" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
     </row>
     <row r="2" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="93" t="s">
+      <c r="B2" s="97"/>
+      <c r="C2" s="106" t="s">
         <v>434</v>
       </c>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="89" t="s">
+      <c r="B3" s="105"/>
+      <c r="C3" s="102" t="s">
         <v>324</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="101" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="87" t="s">
+      <c r="B4" s="101"/>
+      <c r="C4" s="100" t="s">
         <v>433</v>
       </c>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="97" t="s">
+      <c r="A6" s="81" t="s">
         <v>240</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
+      <c r="B6" s="82"/>
+      <c r="C6" s="82"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="82"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="104" t="s">
+      <c r="A7" s="88" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="105"/>
+      <c r="B7" s="89"/>
       <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
@@ -4111,10 +4113,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="26" x14ac:dyDescent="0.2">
-      <c r="A8" s="108">
+      <c r="A8" s="92">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B8" s="109"/>
+      <c r="B8" s="93"/>
       <c r="C8" s="3" t="s">
         <v>25</v>
       </c>
@@ -4122,10 +4124,10 @@
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A9" s="110">
+      <c r="A9" s="94">
         <v>1.2</v>
       </c>
-      <c r="B9" s="111"/>
+      <c r="B9" s="95"/>
       <c r="C9" s="5" t="s">
         <v>26</v>
       </c>
@@ -4133,10 +4135,10 @@
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="26" x14ac:dyDescent="0.2">
-      <c r="A10" s="108">
+      <c r="A10" s="92">
         <v>1.3</v>
       </c>
-      <c r="B10" s="109"/>
+      <c r="B10" s="93"/>
       <c r="C10" s="3" t="s">
         <v>27</v>
       </c>
@@ -4144,10 +4146,10 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="26" x14ac:dyDescent="0.2">
-      <c r="A11" s="110">
+      <c r="A11" s="94">
         <v>1.4</v>
       </c>
-      <c r="B11" s="111"/>
+      <c r="B11" s="95"/>
       <c r="C11" s="5" t="s">
         <v>28</v>
       </c>
@@ -4155,10 +4157,10 @@
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="108">
+      <c r="A12" s="92">
         <v>1.5</v>
       </c>
-      <c r="B12" s="109"/>
+      <c r="B12" s="93"/>
       <c r="C12" s="3" t="s">
         <v>29</v>
       </c>
@@ -4166,32 +4168,32 @@
       <c r="E12" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="81" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
+      <c r="B14" s="82"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="106" t="s">
+      <c r="A15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="102" t="s">
+      <c r="A16" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="103"/>
+      <c r="B16" s="87"/>
       <c r="C16" s="2" t="s">
         <v>31</v>
       </c>
@@ -4243,9 +4245,7 @@
       <c r="E18" s="43" t="s">
         <v>465</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>466</v>
-      </c>
+      <c r="F18" s="6"/>
       <c r="G18" s="5"/>
     </row>
     <row r="19" spans="1:7" ht="172.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -4306,44 +4306,44 @@
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="107" t="s">
+      <c r="A22" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="64"/>
+      <c r="B22" s="73"/>
       <c r="C22" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="8" cm="1">
+      <c r="D22" s="8" t="str" cm="1">
         <f t="array" ref="D22">IFERROR(LOOKUP(2,1/(F17:F21&lt;&gt;""),{1;2;3;4;5}),"")</f>
-        <v>2</v>
-      </c>
-      <c r="E22" s="100" t="s">
+        <v/>
+      </c>
+      <c r="E22" s="84" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="101"/>
-      <c r="G22" s="101"/>
+      <c r="F22" s="85"/>
+      <c r="G22" s="85"/>
     </row>
     <row r="24" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="B24" s="98"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
+      <c r="B24" s="82"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="99" t="s">
+      <c r="A25" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="64"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="64"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
@@ -4420,9 +4420,7 @@
       <c r="E29" s="43" t="s">
         <v>248</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>466</v>
-      </c>
+      <c r="F29" s="6"/>
       <c r="G29" s="5"/>
     </row>
     <row r="30" spans="1:7" ht="120.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4445,166 +4443,194 @@
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="95" t="s">
+      <c r="A31" s="79" t="s">
         <v>109</v>
       </c>
-      <c r="B31" s="64"/>
+      <c r="B31" s="73"/>
       <c r="C31" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="8" cm="1">
+      <c r="D31" s="8" t="str" cm="1">
         <f t="array" ref="D31">IFERROR(LOOKUP(2,1/(F27:F30&lt;&gt;""),{1;2;3;4}),"")</f>
-        <v>3</v>
-      </c>
-      <c r="E31" s="96" t="s">
+        <v/>
+      </c>
+      <c r="E31" s="80" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="33" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="82" t="s">
+      <c r="A33" s="108" t="s">
         <v>266</v>
       </c>
-      <c r="B33" s="82"/>
-      <c r="C33" s="82"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="82"/>
-      <c r="F33" s="82"/>
-      <c r="G33" s="82"/>
+      <c r="B33" s="108"/>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
+      <c r="E33" s="108"/>
+      <c r="F33" s="108"/>
+      <c r="G33" s="108"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="81" t="s">
+      <c r="A34" s="109" t="s">
         <v>261</v>
       </c>
-      <c r="B34" s="81"/>
-      <c r="C34" s="81" t="s">
+      <c r="B34" s="109"/>
+      <c r="C34" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81"/>
-      <c r="G34" s="81"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="109"/>
+      <c r="F34" s="109"/>
+      <c r="G34" s="109"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="79" t="s">
+      <c r="A35" s="110" t="s">
         <v>263</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="80" t="s">
+      <c r="B35" s="110"/>
+      <c r="C35" s="111" t="s">
         <v>269</v>
       </c>
-      <c r="D35" s="80"/>
-      <c r="E35" s="80"/>
-      <c r="F35" s="80"/>
-      <c r="G35" s="80"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="111"/>
+      <c r="F35" s="111"/>
+      <c r="G35" s="111"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="79" t="s">
+      <c r="A36" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="79"/>
-      <c r="C36" s="80" t="s">
+      <c r="B36" s="110"/>
+      <c r="C36" s="111" t="s">
         <v>300</v>
       </c>
-      <c r="D36" s="80"/>
-      <c r="E36" s="80"/>
-      <c r="F36" s="80"/>
-      <c r="G36" s="80"/>
+      <c r="D36" s="111"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="111"/>
+      <c r="G36" s="111"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="79" t="s">
+      <c r="A37" s="110" t="s">
         <v>9</v>
       </c>
-      <c r="B37" s="79"/>
-      <c r="C37" s="80" t="s">
+      <c r="B37" s="110"/>
+      <c r="C37" s="111" t="s">
         <v>301</v>
       </c>
-      <c r="D37" s="80"/>
-      <c r="E37" s="80"/>
-      <c r="F37" s="80"/>
-      <c r="G37" s="80"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="111"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="79" t="s">
+      <c r="A38" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="80" t="s">
+      <c r="B38" s="110"/>
+      <c r="C38" s="111" t="s">
         <v>302</v>
       </c>
-      <c r="D38" s="80"/>
-      <c r="E38" s="80"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="80"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
+      <c r="F38" s="111"/>
+      <c r="G38" s="111"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="81" t="s">
+      <c r="A40" s="109" t="s">
         <v>265</v>
       </c>
-      <c r="B40" s="81"/>
-      <c r="C40" s="81" t="s">
+      <c r="B40" s="109"/>
+      <c r="C40" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="81"/>
+      <c r="D40" s="109"/>
+      <c r="E40" s="109"/>
+      <c r="F40" s="109"/>
+      <c r="G40" s="109"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="79" t="s">
+      <c r="A41" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="79"/>
-      <c r="C41" s="80" t="s">
+      <c r="B41" s="110"/>
+      <c r="C41" s="111" t="s">
         <v>430</v>
       </c>
-      <c r="D41" s="80"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="80"/>
-      <c r="G41" s="80"/>
+      <c r="D41" s="111"/>
+      <c r="E41" s="111"/>
+      <c r="F41" s="111"/>
+      <c r="G41" s="111"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="79" t="s">
+      <c r="A42" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="80" t="s">
+      <c r="B42" s="110"/>
+      <c r="C42" s="111" t="s">
         <v>303</v>
       </c>
-      <c r="D42" s="80"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="80"/>
-      <c r="G42" s="80"/>
+      <c r="D42" s="111"/>
+      <c r="E42" s="111"/>
+      <c r="F42" s="111"/>
+      <c r="G42" s="111"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="79" t="s">
+      <c r="A43" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="80" t="s">
+      <c r="B43" s="110"/>
+      <c r="C43" s="111" t="s">
         <v>304</v>
       </c>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="80"/>
-      <c r="G43" s="80"/>
+      <c r="D43" s="111"/>
+      <c r="E43" s="111"/>
+      <c r="F43" s="111"/>
+      <c r="G43" s="111"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="79" t="s">
+      <c r="A44" s="110" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="79"/>
-      <c r="C44" s="80" t="s">
+      <c r="B44" s="110"/>
+      <c r="C44" s="111" t="s">
         <v>305</v>
       </c>
-      <c r="D44" s="80"/>
-      <c r="E44" s="80"/>
-      <c r="F44" s="80"/>
-      <c r="G44" s="80"/>
+      <c r="D44" s="111"/>
+      <c r="E44" s="111"/>
+      <c r="F44" s="111"/>
+      <c r="G44" s="111"/>
     </row>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C2:G2"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="A6:G6"/>
@@ -4621,34 +4647,6 @@
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C44:G44"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:G42"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
   <dataValidations count="2">
@@ -4681,71 +4679,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="119" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
     </row>
     <row r="2" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="93" t="s">
+      <c r="B2" s="97"/>
+      <c r="C2" s="106" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
     </row>
     <row r="3" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="89" t="s">
+      <c r="B3" s="105"/>
+      <c r="C3" s="102" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
     </row>
     <row r="4" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="101" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="87" t="s">
+      <c r="B4" s="101"/>
+      <c r="C4" s="100" t="s">
         <v>112</v>
       </c>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="97" t="s">
+      <c r="A6" s="81" t="s">
         <v>239</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
+      <c r="B6" s="82"/>
+      <c r="C6" s="82"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="82"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="118" t="s">
+      <c r="A7" s="113" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="119"/>
+      <c r="B7" s="114"/>
       <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
@@ -4757,10 +4755,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="113">
+      <c r="A8" s="115">
         <v>2.1</v>
       </c>
-      <c r="B8" s="114"/>
+      <c r="B8" s="116"/>
       <c r="C8" s="42" t="s">
         <v>113</v>
       </c>
@@ -4768,10 +4766,10 @@
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="57.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="115">
+      <c r="A9" s="117">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B9" s="116"/>
+      <c r="B9" s="118"/>
       <c r="C9" s="31" t="s">
         <v>114</v>
       </c>
@@ -4779,10 +4777,10 @@
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="113">
+      <c r="A10" s="115">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B10" s="114"/>
+      <c r="B10" s="116"/>
       <c r="C10" s="42" t="s">
         <v>115</v>
       </c>
@@ -4790,10 +4788,10 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="115">
+      <c r="A11" s="117">
         <v>2.4</v>
       </c>
-      <c r="B11" s="116"/>
+      <c r="B11" s="118"/>
       <c r="C11" s="31" t="s">
         <v>116</v>
       </c>
@@ -4801,10 +4799,10 @@
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="113">
+      <c r="A12" s="115">
         <v>2.5</v>
       </c>
-      <c r="B12" s="114"/>
+      <c r="B12" s="116"/>
       <c r="C12" s="42" t="s">
         <v>117</v>
       </c>
@@ -4812,32 +4810,32 @@
       <c r="E12" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="81" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
+      <c r="B14" s="82"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="106" t="s">
+      <c r="A15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="102" t="s">
+      <c r="A16" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="103"/>
+      <c r="B16" s="87"/>
       <c r="C16" s="2" t="s">
         <v>31</v>
       </c>
@@ -4950,10 +4948,10 @@
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="95" t="s">
+      <c r="A22" s="79" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="64"/>
+      <c r="B22" s="73"/>
       <c r="C22" s="7" t="s">
         <v>36</v>
       </c>
@@ -4961,39 +4959,39 @@
         <f t="array" ref="D22">IFERROR(LOOKUP(2,1/(F17:F21&lt;&gt;""),{1;2;3;4;5}),"")</f>
         <v/>
       </c>
-      <c r="E22" s="117" t="s">
+      <c r="E22" s="112" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="64"/>
-      <c r="G22" s="64"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="73"/>
     </row>
     <row r="24" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="B24" s="98"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
+      <c r="B24" s="82"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="106" t="s">
+      <c r="A25" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="64"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="64"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="102" t="s">
+      <c r="A26" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="103"/>
+      <c r="B26" s="87"/>
       <c r="C26" s="30" t="s">
         <v>143</v>
       </c>
@@ -5087,10 +5085,10 @@
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="107" t="s">
+      <c r="A31" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="64"/>
+      <c r="B31" s="73"/>
       <c r="C31" s="44" t="s">
         <v>41</v>
       </c>
@@ -5098,166 +5096,173 @@
         <f t="array" ref="D31">IFERROR(LOOKUP(2,1/(F27:F30&lt;&gt;""),{1;2;3;4}),"")</f>
         <v/>
       </c>
-      <c r="E31" s="117" t="s">
+      <c r="E31" s="112" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="33" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="82" t="s">
+      <c r="A33" s="108" t="s">
         <v>266</v>
       </c>
-      <c r="B33" s="82"/>
-      <c r="C33" s="82"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="82"/>
-      <c r="F33" s="82"/>
-      <c r="G33" s="82"/>
+      <c r="B33" s="108"/>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
+      <c r="E33" s="108"/>
+      <c r="F33" s="108"/>
+      <c r="G33" s="108"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="81" t="s">
+      <c r="A34" s="109" t="s">
         <v>261</v>
       </c>
-      <c r="B34" s="81"/>
-      <c r="C34" s="81" t="s">
+      <c r="B34" s="109"/>
+      <c r="C34" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81"/>
-      <c r="G34" s="81"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="109"/>
+      <c r="F34" s="109"/>
+      <c r="G34" s="109"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="79" t="s">
+      <c r="A35" s="110" t="s">
         <v>263</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="80" t="s">
+      <c r="B35" s="110"/>
+      <c r="C35" s="111" t="s">
         <v>268</v>
       </c>
-      <c r="D35" s="80"/>
-      <c r="E35" s="80"/>
-      <c r="F35" s="80"/>
-      <c r="G35" s="80"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="111"/>
+      <c r="F35" s="111"/>
+      <c r="G35" s="111"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="79" t="s">
+      <c r="A36" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="79"/>
-      <c r="C36" s="80" t="s">
+      <c r="B36" s="110"/>
+      <c r="C36" s="111" t="s">
         <v>293</v>
       </c>
-      <c r="D36" s="80"/>
-      <c r="E36" s="80"/>
-      <c r="F36" s="80"/>
-      <c r="G36" s="80"/>
+      <c r="D36" s="111"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="111"/>
+      <c r="G36" s="111"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="79" t="s">
+      <c r="A37" s="110" t="s">
         <v>9</v>
       </c>
-      <c r="B37" s="79"/>
-      <c r="C37" s="80" t="s">
+      <c r="B37" s="110"/>
+      <c r="C37" s="111" t="s">
         <v>294</v>
       </c>
-      <c r="D37" s="80"/>
-      <c r="E37" s="80"/>
-      <c r="F37" s="80"/>
-      <c r="G37" s="80"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="111"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="79" t="s">
+      <c r="A38" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="80" t="s">
+      <c r="B38" s="110"/>
+      <c r="C38" s="111" t="s">
         <v>295</v>
       </c>
-      <c r="D38" s="80"/>
-      <c r="E38" s="80"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="80"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
+      <c r="F38" s="111"/>
+      <c r="G38" s="111"/>
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="81" t="s">
+      <c r="A40" s="109" t="s">
         <v>265</v>
       </c>
-      <c r="B40" s="81"/>
-      <c r="C40" s="81" t="s">
+      <c r="B40" s="109"/>
+      <c r="C40" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="81"/>
+      <c r="D40" s="109"/>
+      <c r="E40" s="109"/>
+      <c r="F40" s="109"/>
+      <c r="G40" s="109"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="79" t="s">
+      <c r="A41" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="79"/>
-      <c r="C41" s="80" t="s">
+      <c r="B41" s="110"/>
+      <c r="C41" s="111" t="s">
         <v>296</v>
       </c>
-      <c r="D41" s="80"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="80"/>
-      <c r="G41" s="80"/>
+      <c r="D41" s="111"/>
+      <c r="E41" s="111"/>
+      <c r="F41" s="111"/>
+      <c r="G41" s="111"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="79" t="s">
+      <c r="A42" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="80" t="s">
+      <c r="B42" s="110"/>
+      <c r="C42" s="111" t="s">
         <v>297</v>
       </c>
-      <c r="D42" s="80"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="80"/>
-      <c r="G42" s="80"/>
+      <c r="D42" s="111"/>
+      <c r="E42" s="111"/>
+      <c r="F42" s="111"/>
+      <c r="G42" s="111"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="79" t="s">
+      <c r="A43" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="80" t="s">
+      <c r="B43" s="110"/>
+      <c r="C43" s="111" t="s">
         <v>298</v>
       </c>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="80"/>
-      <c r="G43" s="80"/>
+      <c r="D43" s="111"/>
+      <c r="E43" s="111"/>
+      <c r="F43" s="111"/>
+      <c r="G43" s="111"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="79" t="s">
+      <c r="A44" s="110" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="79"/>
-      <c r="C44" s="80" t="s">
+      <c r="B44" s="110"/>
+      <c r="C44" s="111" t="s">
         <v>299</v>
       </c>
-      <c r="D44" s="80"/>
-      <c r="E44" s="80"/>
-      <c r="F44" s="80"/>
-      <c r="G44" s="80"/>
+      <c r="D44" s="111"/>
+      <c r="E44" s="111"/>
+      <c r="F44" s="111"/>
+      <c r="G44" s="111"/>
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:G37"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A16:B16"/>
@@ -5274,24 +5279,17 @@
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D8:D12" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -5323,54 +5321,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="119" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
     </row>
     <row r="2" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="93" t="s">
+      <c r="B2" s="97"/>
+      <c r="C2" s="106" t="s">
         <v>144</v>
       </c>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
     </row>
     <row r="3" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="89" t="s">
+      <c r="B3" s="105"/>
+      <c r="C3" s="102" t="s">
         <v>145</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
     </row>
     <row r="4" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="101" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="87" t="s">
+      <c r="B4" s="101"/>
+      <c r="C4" s="100" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="120" t="s">
@@ -5382,10 +5380,10 @@
       <c r="E6" s="120"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="118" t="s">
+      <c r="A7" s="113" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="119"/>
+      <c r="B7" s="114"/>
       <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
@@ -5397,10 +5395,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="52" x14ac:dyDescent="0.2">
-      <c r="A8" s="113">
+      <c r="A8" s="115">
         <v>3.1</v>
       </c>
-      <c r="B8" s="114"/>
+      <c r="B8" s="116"/>
       <c r="C8" s="42" t="s">
         <v>147</v>
       </c>
@@ -5408,10 +5406,10 @@
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A9" s="115">
+      <c r="A9" s="117">
         <v>3.2</v>
       </c>
-      <c r="B9" s="116"/>
+      <c r="B9" s="118"/>
       <c r="C9" s="5" t="s">
         <v>148</v>
       </c>
@@ -5419,10 +5417,10 @@
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A10" s="113">
+      <c r="A10" s="115">
         <v>3.3</v>
       </c>
-      <c r="B10" s="114"/>
+      <c r="B10" s="116"/>
       <c r="C10" s="42" t="s">
         <v>149</v>
       </c>
@@ -5430,10 +5428,10 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A11" s="115">
+      <c r="A11" s="117">
         <v>3.4</v>
       </c>
-      <c r="B11" s="116"/>
+      <c r="B11" s="118"/>
       <c r="C11" s="31" t="s">
         <v>47</v>
       </c>
@@ -5441,10 +5439,10 @@
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="52" x14ac:dyDescent="0.2">
-      <c r="A12" s="113">
+      <c r="A12" s="115">
         <v>3.5</v>
       </c>
-      <c r="B12" s="114"/>
+      <c r="B12" s="116"/>
       <c r="C12" s="42" t="s">
         <v>150</v>
       </c>
@@ -5452,32 +5450,32 @@
       <c r="E12" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="81" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
+      <c r="B14" s="82"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="106" t="s">
+      <c r="A15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="102" t="s">
+      <c r="A16" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="103"/>
+      <c r="B16" s="87"/>
       <c r="C16" s="2" t="s">
         <v>31</v>
       </c>
@@ -5590,10 +5588,10 @@
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="107" t="s">
+      <c r="A22" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="64"/>
+      <c r="B22" s="73"/>
       <c r="C22" s="7" t="s">
         <v>36</v>
       </c>
@@ -5601,39 +5599,39 @@
         <f t="array" ref="D22">IFERROR(LOOKUP(2,1/(F17:F21&lt;&gt;""),{1;2;3;4;5}),"")</f>
         <v/>
       </c>
-      <c r="E22" s="96" t="s">
+      <c r="E22" s="80" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="64"/>
-      <c r="G22" s="64"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="73"/>
     </row>
     <row r="24" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="B24" s="98"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
+      <c r="B24" s="82"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="99" t="s">
+      <c r="A25" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="64"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="64"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="102" t="s">
+      <c r="A26" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="103"/>
+      <c r="B26" s="87"/>
       <c r="C26" s="30" t="s">
         <v>143</v>
       </c>
@@ -5727,10 +5725,10 @@
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="107" t="s">
+      <c r="A31" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="64"/>
+      <c r="B31" s="73"/>
       <c r="C31" s="7" t="s">
         <v>41</v>
       </c>
@@ -5738,166 +5736,173 @@
         <f t="array" ref="D31">IFERROR(LOOKUP(2,1/(F27:F30&lt;&gt;""),{1;2;3;4}),"")</f>
         <v/>
       </c>
-      <c r="E31" s="96" t="s">
+      <c r="E31" s="80" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="33" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="82" t="s">
+      <c r="A33" s="108" t="s">
         <v>266</v>
       </c>
-      <c r="B33" s="82"/>
-      <c r="C33" s="82"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="82"/>
-      <c r="F33" s="82"/>
-      <c r="G33" s="82"/>
+      <c r="B33" s="108"/>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
+      <c r="E33" s="108"/>
+      <c r="F33" s="108"/>
+      <c r="G33" s="108"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="81" t="s">
+      <c r="A34" s="109" t="s">
         <v>261</v>
       </c>
-      <c r="B34" s="81"/>
-      <c r="C34" s="81" t="s">
+      <c r="B34" s="109"/>
+      <c r="C34" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81"/>
-      <c r="G34" s="81"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="109"/>
+      <c r="F34" s="109"/>
+      <c r="G34" s="109"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="79" t="s">
+      <c r="A35" s="110" t="s">
         <v>263</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="80" t="s">
+      <c r="B35" s="110"/>
+      <c r="C35" s="111" t="s">
         <v>267</v>
       </c>
-      <c r="D35" s="80"/>
-      <c r="E35" s="80"/>
-      <c r="F35" s="80"/>
-      <c r="G35" s="80"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="111"/>
+      <c r="F35" s="111"/>
+      <c r="G35" s="111"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="79" t="s">
+      <c r="A36" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="79"/>
-      <c r="C36" s="80" t="s">
+      <c r="B36" s="110"/>
+      <c r="C36" s="111" t="s">
         <v>286</v>
       </c>
-      <c r="D36" s="80"/>
-      <c r="E36" s="80"/>
-      <c r="F36" s="80"/>
-      <c r="G36" s="80"/>
+      <c r="D36" s="111"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="111"/>
+      <c r="G36" s="111"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="79" t="s">
+      <c r="A37" s="110" t="s">
         <v>9</v>
       </c>
-      <c r="B37" s="79"/>
-      <c r="C37" s="80" t="s">
+      <c r="B37" s="110"/>
+      <c r="C37" s="111" t="s">
         <v>287</v>
       </c>
-      <c r="D37" s="80"/>
-      <c r="E37" s="80"/>
-      <c r="F37" s="80"/>
-      <c r="G37" s="80"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="111"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="79" t="s">
+      <c r="A38" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="80" t="s">
+      <c r="B38" s="110"/>
+      <c r="C38" s="111" t="s">
         <v>288</v>
       </c>
-      <c r="D38" s="80"/>
-      <c r="E38" s="80"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="80"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
+      <c r="F38" s="111"/>
+      <c r="G38" s="111"/>
     </row>
     <row r="40" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="81" t="s">
+      <c r="A40" s="109" t="s">
         <v>265</v>
       </c>
-      <c r="B40" s="81"/>
-      <c r="C40" s="81" t="s">
+      <c r="B40" s="109"/>
+      <c r="C40" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="81"/>
+      <c r="D40" s="109"/>
+      <c r="E40" s="109"/>
+      <c r="F40" s="109"/>
+      <c r="G40" s="109"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="79" t="s">
+      <c r="A41" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="79"/>
-      <c r="C41" s="80" t="s">
+      <c r="B41" s="110"/>
+      <c r="C41" s="111" t="s">
         <v>289</v>
       </c>
-      <c r="D41" s="80"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="80"/>
-      <c r="G41" s="80"/>
+      <c r="D41" s="111"/>
+      <c r="E41" s="111"/>
+      <c r="F41" s="111"/>
+      <c r="G41" s="111"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="79" t="s">
+      <c r="A42" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="80" t="s">
+      <c r="B42" s="110"/>
+      <c r="C42" s="111" t="s">
         <v>290</v>
       </c>
-      <c r="D42" s="80"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="80"/>
-      <c r="G42" s="80"/>
+      <c r="D42" s="111"/>
+      <c r="E42" s="111"/>
+      <c r="F42" s="111"/>
+      <c r="G42" s="111"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="79" t="s">
+      <c r="A43" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="80" t="s">
+      <c r="B43" s="110"/>
+      <c r="C43" s="111" t="s">
         <v>291</v>
       </c>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="80"/>
-      <c r="G43" s="80"/>
+      <c r="D43" s="111"/>
+      <c r="E43" s="111"/>
+      <c r="F43" s="111"/>
+      <c r="G43" s="111"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="79" t="s">
+      <c r="A44" s="110" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="79"/>
-      <c r="C44" s="80" t="s">
+      <c r="B44" s="110"/>
+      <c r="C44" s="111" t="s">
         <v>292</v>
       </c>
-      <c r="D44" s="80"/>
-      <c r="E44" s="80"/>
-      <c r="F44" s="80"/>
-      <c r="G44" s="80"/>
+      <c r="D44" s="111"/>
+      <c r="E44" s="111"/>
+      <c r="F44" s="111"/>
+      <c r="G44" s="111"/>
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:G37"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A16:B16"/>
@@ -5914,24 +5919,17 @@
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="C2:G2"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D8:D12" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -5963,54 +5961,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="98" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
     </row>
     <row r="2" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="93" t="s">
+      <c r="B2" s="97"/>
+      <c r="C2" s="106" t="s">
         <v>171</v>
       </c>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
     </row>
     <row r="3" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="89" t="s">
+      <c r="B3" s="105"/>
+      <c r="C3" s="102" t="s">
         <v>172</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="101" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="87" t="s">
+      <c r="B4" s="101"/>
+      <c r="C4" s="100" t="s">
         <v>173</v>
       </c>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="120" t="s">
@@ -6022,10 +6020,10 @@
       <c r="E6" s="120"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="118" t="s">
+      <c r="A7" s="113" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="119"/>
+      <c r="B7" s="114"/>
       <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
@@ -6037,10 +6035,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A8" s="113">
+      <c r="A8" s="115">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B8" s="114"/>
+      <c r="B8" s="116"/>
       <c r="C8" s="42" t="s">
         <v>174</v>
       </c>
@@ -6048,10 +6046,10 @@
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A9" s="115">
+      <c r="A9" s="117">
         <v>4.2</v>
       </c>
-      <c r="B9" s="116"/>
+      <c r="B9" s="118"/>
       <c r="C9" s="31" t="s">
         <v>175</v>
       </c>
@@ -6059,10 +6057,10 @@
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A10" s="113">
+      <c r="A10" s="115">
         <v>4.3</v>
       </c>
-      <c r="B10" s="114"/>
+      <c r="B10" s="116"/>
       <c r="C10" s="42" t="s">
         <v>176</v>
       </c>
@@ -6070,10 +6068,10 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A11" s="115">
+      <c r="A11" s="117">
         <v>4.4000000000000004</v>
       </c>
-      <c r="B11" s="116"/>
+      <c r="B11" s="118"/>
       <c r="C11" s="31" t="s">
         <v>177</v>
       </c>
@@ -6081,10 +6079,10 @@
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="52" x14ac:dyDescent="0.2">
-      <c r="A12" s="113">
+      <c r="A12" s="115">
         <v>4.5</v>
       </c>
-      <c r="B12" s="114"/>
+      <c r="B12" s="116"/>
       <c r="C12" s="42" t="s">
         <v>178</v>
       </c>
@@ -6092,32 +6090,32 @@
       <c r="E12" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="81" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
+      <c r="B14" s="82"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="106" t="s">
+      <c r="A15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="102" t="s">
+      <c r="A16" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="103"/>
+      <c r="B16" s="87"/>
       <c r="C16" s="2" t="s">
         <v>31</v>
       </c>
@@ -6230,10 +6228,10 @@
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="107" t="s">
+      <c r="A22" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="64"/>
+      <c r="B22" s="73"/>
       <c r="C22" s="7" t="s">
         <v>36</v>
       </c>
@@ -6241,39 +6239,39 @@
         <f t="array" ref="D22">IFERROR(LOOKUP(2,1/(F17:F21&lt;&gt;""),{1;2;3;4;5}),"")</f>
         <v/>
       </c>
-      <c r="E22" s="117" t="s">
+      <c r="E22" s="112" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="64"/>
-      <c r="G22" s="64"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="73"/>
     </row>
     <row r="24" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="B24" s="98"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
+      <c r="B24" s="82"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="106" t="s">
+      <c r="A25" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="64"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="64"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="102" t="s">
+      <c r="A26" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="103"/>
+      <c r="B26" s="87"/>
       <c r="C26" s="30" t="s">
         <v>143</v>
       </c>
@@ -6367,10 +6365,10 @@
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="107" t="s">
+      <c r="A31" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="64"/>
+      <c r="B31" s="73"/>
       <c r="C31" s="7" t="s">
         <v>41</v>
       </c>
@@ -6378,155 +6376,184 @@
         <f t="array" ref="D31">IFERROR(LOOKUP(2,1/(F27:F30&lt;&gt;""),{1;2;3;4}),"")</f>
         <v/>
       </c>
-      <c r="E31" s="117" t="s">
+      <c r="E31" s="112" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="34" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="82" t="s">
+      <c r="A34" s="108" t="s">
         <v>266</v>
       </c>
-      <c r="B34" s="82"/>
-      <c r="C34" s="82"/>
-      <c r="D34" s="82"/>
-      <c r="E34" s="82"/>
-      <c r="F34" s="82"/>
-      <c r="G34" s="82"/>
+      <c r="B34" s="108"/>
+      <c r="C34" s="108"/>
+      <c r="D34" s="108"/>
+      <c r="E34" s="108"/>
+      <c r="F34" s="108"/>
+      <c r="G34" s="108"/>
     </row>
     <row r="35" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="81" t="s">
+      <c r="A35" s="109" t="s">
         <v>261</v>
       </c>
-      <c r="B35" s="81"/>
-      <c r="C35" s="81" t="s">
+      <c r="B35" s="109"/>
+      <c r="C35" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D35" s="81"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="81"/>
-      <c r="G35" s="81"/>
+      <c r="D35" s="109"/>
+      <c r="E35" s="109"/>
+      <c r="F35" s="109"/>
+      <c r="G35" s="109"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="79" t="s">
+      <c r="A36" s="110" t="s">
         <v>263</v>
       </c>
-      <c r="B36" s="79"/>
-      <c r="C36" s="80" t="s">
+      <c r="B36" s="110"/>
+      <c r="C36" s="111" t="s">
         <v>264</v>
       </c>
-      <c r="D36" s="80"/>
-      <c r="E36" s="80"/>
-      <c r="F36" s="80"/>
-      <c r="G36" s="80"/>
+      <c r="D36" s="111"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="111"/>
+      <c r="G36" s="111"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="79" t="s">
+      <c r="A37" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="B37" s="79"/>
-      <c r="C37" s="80" t="s">
+      <c r="B37" s="110"/>
+      <c r="C37" s="111" t="s">
         <v>279</v>
       </c>
-      <c r="D37" s="80"/>
-      <c r="E37" s="80"/>
-      <c r="F37" s="80"/>
-      <c r="G37" s="80"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="111"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="79" t="s">
+      <c r="A38" s="110" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="80" t="s">
+      <c r="B38" s="110"/>
+      <c r="C38" s="111" t="s">
         <v>280</v>
       </c>
-      <c r="D38" s="80"/>
-      <c r="E38" s="80"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="80"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
+      <c r="F38" s="111"/>
+      <c r="G38" s="111"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="79" t="s">
+      <c r="A39" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="79"/>
-      <c r="C39" s="80" t="s">
+      <c r="B39" s="110"/>
+      <c r="C39" s="111" t="s">
         <v>281</v>
       </c>
-      <c r="D39" s="80"/>
-      <c r="E39" s="80"/>
-      <c r="F39" s="80"/>
-      <c r="G39" s="80"/>
+      <c r="D39" s="111"/>
+      <c r="E39" s="111"/>
+      <c r="F39" s="111"/>
+      <c r="G39" s="111"/>
     </row>
     <row r="41" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="81" t="s">
+      <c r="A41" s="109" t="s">
         <v>265</v>
       </c>
-      <c r="B41" s="81"/>
-      <c r="C41" s="81" t="s">
+      <c r="B41" s="109"/>
+      <c r="C41" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D41" s="81"/>
-      <c r="E41" s="81"/>
-      <c r="F41" s="81"/>
-      <c r="G41" s="81"/>
+      <c r="D41" s="109"/>
+      <c r="E41" s="109"/>
+      <c r="F41" s="109"/>
+      <c r="G41" s="109"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="79" t="s">
+      <c r="A42" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="80" t="s">
+      <c r="B42" s="110"/>
+      <c r="C42" s="111" t="s">
         <v>282</v>
       </c>
-      <c r="D42" s="80"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="80"/>
-      <c r="G42" s="80"/>
+      <c r="D42" s="111"/>
+      <c r="E42" s="111"/>
+      <c r="F42" s="111"/>
+      <c r="G42" s="111"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="79" t="s">
+      <c r="A43" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="80" t="s">
+      <c r="B43" s="110"/>
+      <c r="C43" s="111" t="s">
         <v>283</v>
       </c>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="80"/>
-      <c r="G43" s="80"/>
+      <c r="D43" s="111"/>
+      <c r="E43" s="111"/>
+      <c r="F43" s="111"/>
+      <c r="G43" s="111"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="79" t="s">
+      <c r="A44" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="B44" s="79"/>
-      <c r="C44" s="80" t="s">
+      <c r="B44" s="110"/>
+      <c r="C44" s="111" t="s">
         <v>284</v>
       </c>
-      <c r="D44" s="80"/>
-      <c r="E44" s="80"/>
-      <c r="F44" s="80"/>
-      <c r="G44" s="80"/>
+      <c r="D44" s="111"/>
+      <c r="E44" s="111"/>
+      <c r="F44" s="111"/>
+      <c r="G44" s="111"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="79" t="s">
+      <c r="A45" s="110" t="s">
         <v>72</v>
       </c>
-      <c r="B45" s="79"/>
-      <c r="C45" s="80" t="s">
+      <c r="B45" s="110"/>
+      <c r="C45" s="111" t="s">
         <v>285</v>
       </c>
-      <c r="D45" s="80"/>
-      <c r="E45" s="80"/>
-      <c r="F45" s="80"/>
-      <c r="G45" s="80"/>
+      <c r="D45" s="111"/>
+      <c r="E45" s="111"/>
+      <c r="F45" s="111"/>
+      <c r="G45" s="111"/>
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:G45"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A6:E6"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="E31:G31"/>
@@ -6543,35 +6570,6 @@
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C44:G44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C45:G45"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:G43"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D8:D12" xr:uid="{00000000-0002-0000-0400-000000000000}">
@@ -6603,54 +6601,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="119" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
     </row>
     <row r="2" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="96" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="121"/>
-      <c r="C2" s="93" t="s">
+      <c r="B2" s="123"/>
+      <c r="C2" s="106" t="s">
         <v>205</v>
       </c>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
     </row>
     <row r="3" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="91" t="s">
+      <c r="A3" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="122"/>
-      <c r="C3" s="89" t="s">
+      <c r="B3" s="121"/>
+      <c r="C3" s="102" t="s">
         <v>206</v>
       </c>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
+      <c r="D3" s="122"/>
+      <c r="E3" s="122"/>
+      <c r="F3" s="122"/>
+      <c r="G3" s="122"/>
     </row>
     <row r="4" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="101" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="87" t="s">
+      <c r="B4" s="101"/>
+      <c r="C4" s="100" t="s">
         <v>207</v>
       </c>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
     </row>
     <row r="6" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="120" t="s">
@@ -6662,10 +6660,10 @@
       <c r="E6" s="120"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="118" t="s">
+      <c r="A7" s="113" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="103"/>
+      <c r="B7" s="87"/>
       <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
@@ -6677,10 +6675,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A8" s="113">
+      <c r="A8" s="115">
         <v>5.0999999999999996</v>
       </c>
-      <c r="B8" s="114"/>
+      <c r="B8" s="116"/>
       <c r="C8" s="42" t="s">
         <v>209</v>
       </c>
@@ -6688,10 +6686,10 @@
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:7" ht="52" x14ac:dyDescent="0.2">
-      <c r="A9" s="115">
+      <c r="A9" s="117">
         <v>5.2</v>
       </c>
-      <c r="B9" s="116"/>
+      <c r="B9" s="118"/>
       <c r="C9" s="31" t="s">
         <v>210</v>
       </c>
@@ -6699,10 +6697,10 @@
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A10" s="113">
+      <c r="A10" s="115">
         <v>5.3</v>
       </c>
-      <c r="B10" s="114"/>
+      <c r="B10" s="116"/>
       <c r="C10" s="42" t="s">
         <v>211</v>
       </c>
@@ -6710,10 +6708,10 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="52" x14ac:dyDescent="0.2">
-      <c r="A11" s="115">
+      <c r="A11" s="117">
         <v>5.4</v>
       </c>
-      <c r="B11" s="116"/>
+      <c r="B11" s="118"/>
       <c r="C11" s="31" t="s">
         <v>438</v>
       </c>
@@ -6721,10 +6719,10 @@
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="39" x14ac:dyDescent="0.2">
-      <c r="A12" s="113">
+      <c r="A12" s="115">
         <v>5.5</v>
       </c>
-      <c r="B12" s="114"/>
+      <c r="B12" s="116"/>
       <c r="C12" s="42" t="s">
         <v>439</v>
       </c>
@@ -6732,32 +6730,32 @@
       <c r="E12" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="97" t="s">
+      <c r="A14" s="81" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
+      <c r="B14" s="82"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="82"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="106" t="s">
+      <c r="A15" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
     </row>
     <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="102" t="s">
+      <c r="A16" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="103"/>
+      <c r="B16" s="87"/>
       <c r="C16" s="2" t="s">
         <v>31</v>
       </c>
@@ -6870,10 +6868,10 @@
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="107" t="s">
+      <c r="A22" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="64"/>
+      <c r="B22" s="73"/>
       <c r="C22" s="7" t="s">
         <v>36</v>
       </c>
@@ -6881,39 +6879,39 @@
         <f t="array" ref="D22">IFERROR(LOOKUP(2,1/(F17:F21&lt;&gt;""),{1;2;3;4;5}),"")</f>
         <v/>
       </c>
-      <c r="E22" s="117" t="s">
+      <c r="E22" s="112" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="64"/>
-      <c r="G22" s="64"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="73"/>
     </row>
     <row r="24" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="97" t="s">
+      <c r="A24" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="B24" s="98"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
+      <c r="B24" s="82"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="106" t="s">
+      <c r="A25" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="64"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="64"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="73"/>
     </row>
     <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="102" t="s">
+      <c r="A26" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="103"/>
+      <c r="B26" s="87"/>
       <c r="C26" s="30" t="s">
         <v>143</v>
       </c>
@@ -7007,10 +7005,10 @@
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="107" t="s">
+      <c r="A31" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="64"/>
+      <c r="B31" s="73"/>
       <c r="C31" s="44" t="s">
         <v>41</v>
       </c>
@@ -7018,155 +7016,184 @@
         <f t="array" ref="D31">IFERROR(LOOKUP(2,1/(F27:F30&lt;&gt;""),{1;2;3;4}),"")</f>
         <v/>
       </c>
-      <c r="E31" s="117" t="s">
+      <c r="E31" s="112" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="33" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="82" t="s">
+      <c r="A33" s="108" t="s">
         <v>271</v>
       </c>
-      <c r="B33" s="82"/>
-      <c r="C33" s="82"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="82"/>
-      <c r="F33" s="82"/>
-      <c r="G33" s="82"/>
+      <c r="B33" s="108"/>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
+      <c r="E33" s="108"/>
+      <c r="F33" s="108"/>
+      <c r="G33" s="108"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="81" t="s">
+      <c r="A34" s="109" t="s">
         <v>261</v>
       </c>
-      <c r="B34" s="81"/>
-      <c r="C34" s="81" t="s">
+      <c r="B34" s="109"/>
+      <c r="C34" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81"/>
-      <c r="G34" s="81"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="109"/>
+      <c r="F34" s="109"/>
+      <c r="G34" s="109"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="79" t="s">
+      <c r="A35" s="110" t="s">
         <v>263</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="80" t="s">
+      <c r="B35" s="110"/>
+      <c r="C35" s="111" t="s">
         <v>270</v>
       </c>
-      <c r="D35" s="80"/>
-      <c r="E35" s="80"/>
-      <c r="F35" s="80"/>
-      <c r="G35" s="80"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="111"/>
+      <c r="F35" s="111"/>
+      <c r="G35" s="111"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="79" t="s">
+      <c r="A36" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="79"/>
-      <c r="C36" s="80" t="s">
+      <c r="B36" s="110"/>
+      <c r="C36" s="111" t="s">
         <v>272</v>
       </c>
-      <c r="D36" s="80"/>
-      <c r="E36" s="80"/>
-      <c r="F36" s="80"/>
-      <c r="G36" s="80"/>
+      <c r="D36" s="111"/>
+      <c r="E36" s="111"/>
+      <c r="F36" s="111"/>
+      <c r="G36" s="111"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="79" t="s">
+      <c r="A37" s="110" t="s">
         <v>9</v>
       </c>
-      <c r="B37" s="79"/>
-      <c r="C37" s="80" t="s">
+      <c r="B37" s="110"/>
+      <c r="C37" s="111" t="s">
         <v>273</v>
       </c>
-      <c r="D37" s="80"/>
-      <c r="E37" s="80"/>
-      <c r="F37" s="80"/>
-      <c r="G37" s="80"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="111"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="79" t="s">
+      <c r="A38" s="110" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="80" t="s">
+      <c r="B38" s="110"/>
+      <c r="C38" s="111" t="s">
         <v>274</v>
       </c>
-      <c r="D38" s="80"/>
-      <c r="E38" s="80"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="80"/>
+      <c r="D38" s="111"/>
+      <c r="E38" s="111"/>
+      <c r="F38" s="111"/>
+      <c r="G38" s="111"/>
     </row>
     <row r="40" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="81" t="s">
+      <c r="A40" s="109" t="s">
         <v>265</v>
       </c>
-      <c r="B40" s="81"/>
-      <c r="C40" s="81" t="s">
+      <c r="B40" s="109"/>
+      <c r="C40" s="109" t="s">
         <v>262</v>
       </c>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="81"/>
+      <c r="D40" s="109"/>
+      <c r="E40" s="109"/>
+      <c r="F40" s="109"/>
+      <c r="G40" s="109"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="79" t="s">
+      <c r="A41" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="79"/>
-      <c r="C41" s="80" t="s">
+      <c r="B41" s="110"/>
+      <c r="C41" s="111" t="s">
         <v>275</v>
       </c>
-      <c r="D41" s="80"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="80"/>
-      <c r="G41" s="80"/>
+      <c r="D41" s="111"/>
+      <c r="E41" s="111"/>
+      <c r="F41" s="111"/>
+      <c r="G41" s="111"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="79" t="s">
+      <c r="A42" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="79"/>
-      <c r="C42" s="80" t="s">
+      <c r="B42" s="110"/>
+      <c r="C42" s="111" t="s">
         <v>276</v>
       </c>
-      <c r="D42" s="80"/>
-      <c r="E42" s="80"/>
-      <c r="F42" s="80"/>
-      <c r="G42" s="80"/>
+      <c r="D42" s="111"/>
+      <c r="E42" s="111"/>
+      <c r="F42" s="111"/>
+      <c r="G42" s="111"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="79" t="s">
+      <c r="A43" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="80" t="s">
+      <c r="B43" s="110"/>
+      <c r="C43" s="111" t="s">
         <v>277</v>
       </c>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="80"/>
-      <c r="G43" s="80"/>
+      <c r="D43" s="111"/>
+      <c r="E43" s="111"/>
+      <c r="F43" s="111"/>
+      <c r="G43" s="111"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="79" t="s">
+      <c r="A44" s="110" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="79"/>
-      <c r="C44" s="80" t="s">
+      <c r="B44" s="110"/>
+      <c r="C44" s="111" t="s">
         <v>278</v>
       </c>
-      <c r="D44" s="80"/>
-      <c r="E44" s="80"/>
-      <c r="F44" s="80"/>
-      <c r="G44" s="80"/>
+      <c r="D44" s="111"/>
+      <c r="E44" s="111"/>
+      <c r="F44" s="111"/>
+      <c r="G44" s="111"/>
     </row>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="E31:G31"/>
@@ -7183,35 +7210,6 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="C44:G44"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:G42"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="D8:D12" xr:uid="{00000000-0002-0000-0500-000000000000}">
@@ -7246,11 +7244,11 @@
       <c r="A1" s="126" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
     </row>
     <row r="2" spans="1:6" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="131" t="s">
@@ -7289,13 +7287,13 @@
       <c r="B5" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="8" t="str">
         <f>'C1'!D22</f>
-        <v>2</v>
-      </c>
-      <c r="D5" s="8">
+        <v/>
+      </c>
+      <c r="D5" s="8" t="str">
         <f>'C1'!D31</f>
-        <v>3</v>
+        <v/>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
@@ -7386,16 +7384,16 @@
       <c r="A12" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="13" t="e">
         <f>AVERAGE(C5:C9)</f>
-        <v>2</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="13" t="e">
         <f>AVERAGE(D5:D9)</f>
-        <v>3</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>